<commit_message>
sync ReactiveSoluteTransport workspace snapshot
</commit_message>
<xml_diff>
--- a/test_case_matrix.xlsx
+++ b/test_case_matrix.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25695" windowHeight="11250"/>
+    <workbookView windowWidth="28800" windowHeight="12975"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Cases" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
     <t>标准设置：V = 1E-4, Np = 1E6, tg = 100 s</t>
   </si>
   <si>
-    <t>Test编号</t>
+    <t xml:space="preserve">Test Case </t>
   </si>
   <si>
     <t>Pressure</t>
@@ -1302,7 +1302,7 @@
         <v>0.0001</v>
       </c>
       <c r="C13" s="5">
-        <v>10000000</v>
+        <v>50000</v>
       </c>
       <c r="D13" s="6">
         <v>100</v>
@@ -1322,6 +1322,9 @@
         <v>1000000</v>
       </c>
       <c r="D14" s="9">
+        <v>5</v>
+      </c>
+      <c r="E14">
         <v>1</v>
       </c>
     </row>
@@ -1338,6 +1341,9 @@
       <c r="D15" s="6">
         <v>10</v>
       </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="7" t="s">
@@ -1356,7 +1362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:5">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -1368,6 +1374,9 @@
       </c>
       <c r="D17" s="6">
         <v>1000</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>